<commit_message>
series add in import
</commit_message>
<xml_diff>
--- a/public/templates/pending_report_sample_template.xlsx
+++ b/public/templates/pending_report_sample_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\work\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Aqsa Work\Softlin Tech\newpresence360\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>S.No</t>
   </si>
@@ -71,6 +71,15 @@
   </si>
   <si>
     <t>FAX-3</t>
+  </si>
+  <si>
+    <t>Series</t>
+  </si>
+  <si>
+    <t>Series Code</t>
+  </si>
+  <si>
+    <t>FA</t>
   </si>
 </sst>
 </file>
@@ -178,77 +187,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="31">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -582,25 +521,25 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
-      <tableStyleElement type="wholeTable" dxfId="37"/>
-      <tableStyleElement type="headerRow" dxfId="36"/>
-      <tableStyleElement type="totalRow" dxfId="35"/>
-      <tableStyleElement type="firstColumn" dxfId="34"/>
-      <tableStyleElement type="lastColumn" dxfId="33"/>
-      <tableStyleElement type="firstRowStripe" dxfId="32"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="31"/>
+      <tableStyleElement type="wholeTable" dxfId="30"/>
+      <tableStyleElement type="headerRow" dxfId="29"/>
+      <tableStyleElement type="totalRow" dxfId="28"/>
+      <tableStyleElement type="firstColumn" dxfId="27"/>
+      <tableStyleElement type="lastColumn" dxfId="26"/>
+      <tableStyleElement type="firstRowStripe" dxfId="25"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="24"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
-      <tableStyleElement type="headerRow" dxfId="30"/>
-      <tableStyleElement type="totalRow" dxfId="29"/>
-      <tableStyleElement type="firstRowStripe" dxfId="28"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="27"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="26"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="25"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="24"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="23"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="22"/>
-      <tableStyleElement type="pageFieldValues" dxfId="21"/>
+      <tableStyleElement type="headerRow" dxfId="23"/>
+      <tableStyleElement type="totalRow" dxfId="22"/>
+      <tableStyleElement type="firstRowStripe" dxfId="21"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="20"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="19"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="18"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="17"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="16"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="15"/>
+      <tableStyleElement type="pageFieldValues" dxfId="14"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -872,18 +811,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.5546875" style="9" customWidth="1"/>
     <col min="2" max="2" width="20.109375" customWidth="1"/>
-    <col min="3" max="3" width="21.109375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="23.33203125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="18.6640625" style="9" customWidth="1"/>
+    <col min="3" max="4" width="21.109375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="23.33203125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" style="9" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22.8" customHeight="1">
+    <row r="1" spans="1:7" ht="22.8" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -894,16 +833,19 @@
         <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="29.4" customHeight="1">
+    <row r="2" spans="1:7" ht="29.4" customHeight="1">
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
@@ -914,16 +856,19 @@
         <v>8</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="29.4" customHeight="1">
+    <row r="3" spans="1:7" ht="29.4" customHeight="1">
       <c r="A3" s="7">
         <v>1</v>
       </c>
@@ -934,37 +879,29 @@
         <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="8">
+      <c r="F3" s="8">
         <v>11764.18</v>
       </c>
-      <c r="F3" s="8">
+      <c r="G3" s="8">
         <v>32322</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="29.4" customHeight="1">
-      <c r="A4" s="7">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="8">
-        <v>11764.18</v>
-      </c>
-      <c r="F4" s="8">
-        <v>32322</v>
-      </c>
+    <row r="4" spans="1:7" ht="29.4" customHeight="1">
+      <c r="A4" s="7"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2">
+  <conditionalFormatting sqref="F2">
     <cfRule type="duplicateValues" dxfId="13" priority="8"/>
     <cfRule type="duplicateValues" dxfId="12" priority="9"/>
     <cfRule type="duplicateValues" dxfId="11" priority="10"/>
@@ -973,7 +910,7 @@
     <cfRule type="duplicateValues" dxfId="8" priority="13"/>
     <cfRule type="duplicateValues" dxfId="7" priority="14"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2">
+  <conditionalFormatting sqref="G2">
     <cfRule type="duplicateValues" dxfId="6" priority="1"/>
     <cfRule type="duplicateValues" dxfId="5" priority="2"/>
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>

</xml_diff>

<commit_message>
working on import pending payments
</commit_message>
<xml_diff>
--- a/public/templates/pending_report_sample_template.xlsx
+++ b/public/templates/pending_report_sample_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Aqsa Work\Softlin Tech\newpresence360\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\work\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>S.No</t>
   </si>
@@ -49,18 +49,12 @@
     <t>Ledger Group</t>
   </si>
   <si>
-    <t>Balance</t>
-  </si>
-  <si>
     <t>Settle Amount</t>
   </si>
   <si>
     <t>Name of ledger parent group</t>
   </si>
   <si>
-    <t>Voucher number</t>
-  </si>
-  <si>
     <t>Vendor</t>
   </si>
   <si>
@@ -80,6 +74,9 @@
   </si>
   <si>
     <t>Voucher No.</t>
+  </si>
+  <si>
+    <t>Voucher Number</t>
   </si>
 </sst>
 </file>
@@ -165,9 +162,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -180,84 +174,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="31">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="24">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -521,25 +448,25 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
-      <tableStyleElement type="wholeTable" dxfId="30"/>
-      <tableStyleElement type="headerRow" dxfId="29"/>
-      <tableStyleElement type="totalRow" dxfId="28"/>
-      <tableStyleElement type="firstColumn" dxfId="27"/>
-      <tableStyleElement type="lastColumn" dxfId="26"/>
-      <tableStyleElement type="firstRowStripe" dxfId="25"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="24"/>
+      <tableStyleElement type="wholeTable" dxfId="23"/>
+      <tableStyleElement type="headerRow" dxfId="22"/>
+      <tableStyleElement type="totalRow" dxfId="21"/>
+      <tableStyleElement type="firstColumn" dxfId="20"/>
+      <tableStyleElement type="lastColumn" dxfId="19"/>
+      <tableStyleElement type="firstRowStripe" dxfId="18"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="17"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
-      <tableStyleElement type="headerRow" dxfId="23"/>
-      <tableStyleElement type="totalRow" dxfId="22"/>
-      <tableStyleElement type="firstRowStripe" dxfId="21"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="20"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="19"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="18"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="17"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="16"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="15"/>
-      <tableStyleElement type="pageFieldValues" dxfId="14"/>
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -811,19 +738,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" style="9" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" customWidth="1"/>
-    <col min="3" max="4" width="21.109375" style="4" customWidth="1"/>
-    <col min="5" max="5" width="23.33203125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" style="9" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" style="8" customWidth="1"/>
+    <col min="3" max="4" width="21.109375" style="9" customWidth="1"/>
+    <col min="5" max="5" width="23.33203125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.8" customHeight="1">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:6" ht="22.8" customHeight="1">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -833,84 +759,57 @@
         <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="2" spans="1:7" ht="29.4" customHeight="1">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:6" ht="29.4" customHeight="1">
+      <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="29.4" customHeight="1">
+      <c r="A3" s="6">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="C3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="29.4" customHeight="1">
-      <c r="A3" s="7">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="8">
-        <v>11764.18</v>
-      </c>
-      <c r="G3" s="8">
+      <c r="F3" s="7">
         <v>32322</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="29.4" customHeight="1">
-      <c r="A4" s="7"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2">
-    <cfRule type="duplicateValues" dxfId="13" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="14"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2">
     <cfRule type="duplicateValues" dxfId="6" priority="1"/>
     <cfRule type="duplicateValues" dxfId="5" priority="2"/>
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>

</xml_diff>

<commit_message>
worked on pending payment import points
</commit_message>
<xml_diff>
--- a/public/templates/pending_report_sample_template.xlsx
+++ b/public/templates/pending_report_sample_template.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>S.No</t>
   </si>
@@ -46,19 +46,10 @@
     <t>Ledger Name</t>
   </si>
   <si>
-    <t>Ledger Group</t>
-  </si>
-  <si>
     <t>Settle Amount</t>
   </si>
   <si>
-    <t>Name of ledger parent group</t>
-  </si>
-  <si>
     <t>Vendor</t>
-  </si>
-  <si>
-    <t>Expense Payables</t>
   </si>
   <si>
     <t>FAX-3</t>
@@ -738,17 +729,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.5546875" style="7" customWidth="1"/>
     <col min="2" max="2" width="20.109375" style="8" customWidth="1"/>
-    <col min="3" max="4" width="21.109375" style="9" customWidth="1"/>
-    <col min="5" max="5" width="23.33203125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="18.6640625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" style="9" customWidth="1"/>
+    <col min="4" max="4" width="23.33203125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22.8" customHeight="1">
+    <row r="1" spans="1:5" ht="22.8" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -756,19 +747,16 @@
         <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>5</v>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="29.4" customHeight="1">
+    <row r="2" spans="1:5" ht="29.4" customHeight="1">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
@@ -776,40 +764,37 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>5</v>
+      <c r="E2" s="5" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="29.4" customHeight="1">
+    <row r="3" spans="1:5" ht="29.4" customHeight="1">
       <c r="A3" s="6">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="7">
+        <v>6</v>
+      </c>
+      <c r="E3" s="7">
         <v>32322</v>
       </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="6"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2">
+  <conditionalFormatting sqref="E2">
     <cfRule type="duplicateValues" dxfId="6" priority="1"/>
     <cfRule type="duplicateValues" dxfId="5" priority="2"/>
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>

</xml_diff>